<commit_message>
Upload test pack: every file as .xlsx
The 44 CSV files are now Excel workbooks with the same rows; the four
Micro-segments pairs are one workbook each with a Lead template and a
Signal template sheet. Every file gives the same results as before when
read the way the POC reads Excel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XiLXGU1oR1hNbNccyNpRo1
</commit_message>
<xml_diff>
--- a/test-data/upload-test-pack/Expected_Results.xlsx
+++ b/test-data/upload-test-pack/Expected_Results.xlsx
@@ -595,7 +595,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>4-Micro-segments-and-Review (N01-N04): each is a pair. Upload the "_1_prospects" file as the prospect list, then the "_2_signals" file, then send the scoring to Micro-segments &amp; NBA and open For Review.</t>
+          <t>4-Micro-segments-and-Review (N01-N04): each file holds a "Lead template" and a "Signal template" sheet. Upload it as the prospect list, then drop the same file as the signals; then send the scoring to Micro-segments &amp; NBA and open For Review.</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>P01_clean_list.csv</t>
+          <t>P01_clean_list.xlsx</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P01_clean_list.csv on the upload box.</t>
+          <t>Prospecting: drop P01_clean_list.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>P02_email_problems.csv</t>
+          <t>P02_email_problems.xlsx</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P02_email_problems.csv on the upload box.</t>
+          <t>Prospecting: drop P02_email_problems.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>P03_linkedin_and_no_contact_details.csv</t>
+          <t>P03_linkedin_and_no_contact_details.xlsx</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P03_linkedin_and_no_contact_details.csv on the upload box.</t>
+          <t>Prospecting: drop P03_linkedin_and_no_contact_details.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>P04_duplicates.csv</t>
+          <t>P04_duplicates.xlsx</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P04_duplicates.csv on the upload box.</t>
+          <t>Prospecting: drop P04_duplicates.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>P05_consent_and_opt_out.csv</t>
+          <t>P05_consent_and_opt_out.xlsx</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P05_consent_and_opt_out.csv on the upload box.</t>
+          <t>Prospecting: drop P05_consent_and_opt_out.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>P06_region.csv</t>
+          <t>P06_region.xlsx</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P06_region.csv on the upload box.</t>
+          <t>Prospecting: drop P06_region.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>P07_managed_separately_and_existing_customer.csv</t>
+          <t>P07_managed_separately_and_existing_customer.xlsx</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P07_managed_separately_and_existing_customer.csv on the upload box.</t>
+          <t>Prospecting: drop P07_managed_separately_and_existing_customer.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>P08_company_size_formats.csv</t>
+          <t>P08_company_size_formats.xlsx</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P08_company_size_formats.csv on the upload box.</t>
+          <t>Prospecting: drop P08_company_size_formats.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>P09_account_types.csv</t>
+          <t>P09_account_types.xlsx</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P09_account_types.csv on the upload box.</t>
+          <t>Prospecting: drop P09_account_types.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>P10_industry_classification.csv</t>
+          <t>P10_industry_classification.xlsx</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P10_industry_classification.csv on the upload box.</t>
+          <t>Prospecting: drop P10_industry_classification.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>P11_job_titles_and_persona.csv</t>
+          <t>P11_job_titles_and_persona.xlsx</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P11_job_titles_and_persona.csv on the upload box.</t>
+          <t>Prospecting: drop P11_job_titles_and_persona.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>P12_owner_rep.csv</t>
+          <t>P12_owner_rep.xlsx</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P12_owner_rep.csv on the upload box.</t>
+          <t>Prospecting: drop P12_owner_rep.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>P13_company_details_differ.csv</t>
+          <t>P13_company_details_differ.xlsx</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P13_company_details_differ.csv on the upload box.</t>
+          <t>Prospecting: drop P13_company_details_differ.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>P14_missing_values.csv</t>
+          <t>P14_missing_values.xlsx</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P14_missing_values.csv on the upload box.</t>
+          <t>Prospecting: drop P14_missing_values.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>P15_missing_columns.csv</t>
+          <t>P15_missing_columns.xlsx</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P15_missing_columns.csv on the upload box.</t>
+          <t>Prospecting: drop P15_missing_columns.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>P16_no_company_name_column.csv</t>
+          <t>P16_no_company_name_column.xlsx</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P16_no_company_name_column.csv on the upload box.</t>
+          <t>Prospecting: drop P16_no_company_name_column.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>P17_template_style_headers.csv</t>
+          <t>P17_template_style_headers.xlsx</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P17_template_style_headers.csv.</t>
+          <t>Prospecting: drop P17_template_style_headers.xlsx.</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>P19_wrong_file_signal_file.csv</t>
+          <t>P19_wrong_file_signal_file.xlsx</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P19_wrong_file_signal_file.csv.</t>
+          <t>Prospecting: drop P19_wrong_file_signal_file.xlsx.</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>P20_headers_only.csv</t>
+          <t>P20_headers_only.xlsx</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P20_headers_only.csv.</t>
+          <t>Prospecting: drop P20_headers_only.xlsx.</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>P21_columns_in_another_order.csv</t>
+          <t>P21_columns_in_another_order.xlsx</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P21_columns_in_another_order.csv on the upload box.</t>
+          <t>Prospecting: drop P21_columns_in_another_order.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>P22_commas_quotes_and_accents.csv</t>
+          <t>P22_commas_quotes_and_accents.xlsx</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1894,12 +1894,12 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Values with commas and quotes (quoted in the CSV) and accented names.</t>
+          <t>Values with commas, quotes and accented names.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Prospecting: drop P22_commas_quotes_and_accents.csv on the upload box.</t>
+          <t>Prospecting: drop P22_commas_quotes_and_accents.xlsx on the upload box.</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>S00_prospect_list_for_scoring_and_signals.csv</t>
+          <t>S00_prospect_list_for_scoring_and_signals.xlsx</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>S01_mixed_signals_all_tiers.csv</t>
+          <t>S01_mixed_signals_all_tiers.xlsx</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S01_mixed_signals_all_tiers.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S01_mixed_signals_all_tiers.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>S02_tier_cut_offs.csv</t>
+          <t>S02_tier_cut_offs.xlsx</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S02_tier_cut_offs.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S02_tier_cut_offs.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>S03_same_signal_every_account_fit_effect.csv</t>
+          <t>S03_same_signal_every_account_fit_effect.xlsx</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S03_same_signal_every_account_fit_effect.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S03_same_signal_every_account_fit_effect.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>S04_stacking_several_signals.csv</t>
+          <t>S04_stacking_several_signals.xlsx</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S04_stacking_several_signals.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S04_stacking_several_signals.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>S05_knock_out_installed_system.csv</t>
+          <t>S05_knock_out_installed_system.xlsx</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S05_knock_out_installed_system.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S05_knock_out_installed_system.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>S06_headers_only_no_signals.csv</t>
+          <t>S06_headers_only_no_signals.xlsx</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S06_headers_only_no_signals.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S06_headers_only_no_signals.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>S07_opted_out_person_signal.csv</t>
+          <t>S07_opted_out_person_signal.xlsx</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -2333,7 +2333,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S07_opted_out_person_signal.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop S07_opted_out_person_signal.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>G01_every_signal_type.csv</t>
+          <t>G01_every_signal_type.xlsx</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G01_every_signal_type.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G01_every_signal_type.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>G02_company_matching.csv</t>
+          <t>G02_company_matching.xlsx</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G02_company_matching.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G02_company_matching.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>G03_person_matching.csv</t>
+          <t>G03_person_matching.xlsx</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G03_person_matching.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G03_person_matching.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>G04_dates.csv</t>
+          <t>G04_dates.xlsx</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G04_dates.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G04_dates.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>2 qualified; 6 rejected D3 with the reason. (Note: an Excel file stores real dates, so this test is for CSV files.)</t>
+          <t>2 qualified; 6 rejected D3 with the reason. (The dates are typed as text, as they arrive from a CSV export; G13 has real Excel dates.)</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>G05_signal_type_spelling.csv</t>
+          <t>G05_signal_type_spelling.xlsx</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G05_signal_type_spelling.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G05_signal_type_spelling.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>G06_duplicates.csv</t>
+          <t>G06_duplicates.xlsx</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G06_duplicates.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G06_duplicates.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>G07_stale_window_edges.csv</t>
+          <t>G07_stale_window_edges.xlsx</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G07_stale_window_edges.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G07_stale_window_edges.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>G08_fading_weights.csv</t>
+          <t>G08_fading_weights.xlsx</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G08_fading_weights.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G08_fading_weights.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>G09_missing_detail_and_optional_columns.csv</t>
+          <t>G09_missing_detail_and_optional_columns.xlsx</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -2819,7 +2819,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G09_missing_detail_and_optional_columns.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G09_missing_detail_and_optional_columns.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>G10_missing_detail_column_and_extra_columns.csv</t>
+          <t>G10_missing_detail_column_and_extra_columns.xlsx</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G10_missing_detail_column_and_extra_columns.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G10_missing_detail_column_and_extra_columns.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>G11_no_signal_type_column.csv</t>
+          <t>G11_no_signal_type_column.xlsx</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G11_no_signal_type_column.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G11_no_signal_type_column.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>G12_wrong_file_lead_file.csv</t>
+          <t>G12_wrong_file_lead_file.xlsx</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, drop G12_wrong_file_lead_file.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, drop G12_wrong_file_lead_file.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>G14_signals_for_excluded_and_below_floor_accounts.csv</t>
+          <t>G14_signals_for_excluded_and_below_floor_accounts.xlsx</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G14_signals_for_excluded_and_below_floor_accounts.csv on box 2.</t>
+          <t>Account Scoring: with the S00 list chosen, set "Score as of" to 2026-10-20, then drop G14_signals_for_excluded_and_below_floor_accounts.xlsx on box 2.</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>N01_segment_boundaries_1_prospects.csv + N01_segment_boundaries_2_signals.csv</t>
+          <t>N01_segment_boundaries.xlsx</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: "Upload a prospect file" = N01_segment_boundaries_1_prospects.csv; Score as of 2026-10-20; drop N01_segment_boundaries_2_signals.csv. Then send to Micro-segments &amp; NBA and open For Review.</t>
+          <t>Account Scoring: "Upload a prospect file" = N01_segment_boundaries.xlsx (reads its "Lead template" sheet); Score as of 2026-10-20; drop the same file on box 2 (reads "Signal template"). Then send to Micro-segments &amp; NBA and open For Review.</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>N02_contact_and_channel_1_prospects.csv + N02_contact_and_channel_2_signals.csv</t>
+          <t>N02_contact_and_channel.xlsx</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -3197,7 +3197,7 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: "Upload a prospect file" = N02_contact_and_channel_1_prospects.csv; Score as of 2026-10-20; drop N02_contact_and_channel_2_signals.csv. Then send to Micro-segments &amp; NBA and open For Review.</t>
+          <t>Account Scoring: "Upload a prospect file" = N02_contact_and_channel.xlsx (reads its "Lead template" sheet); Score as of 2026-10-20; drop the same file on box 2 (reads "Signal template"). Then send to Micro-segments &amp; NBA and open For Review.</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>N03_for_review_reasons_1_prospects.csv + N03_for_review_reasons_2_signals.csv</t>
+          <t>N03_for_review_reasons.xlsx</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: "Upload a prospect file" = N03_for_review_reasons_1_prospects.csv; Score as of 2026-10-20; drop N03_for_review_reasons_2_signals.csv. Then send to Micro-segments &amp; NBA and open For Review.</t>
+          <t>Account Scoring: "Upload a prospect file" = N03_for_review_reasons.xlsx (reads its "Lead template" sheet); Score as of 2026-10-20; drop the same file on box 2 (reads "Signal template"). Then send to Micro-segments &amp; NBA and open For Review.</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>N04_rep_ownership_1_prospects.csv + N04_rep_ownership_2_signals.csv</t>
+          <t>N04_rep_ownership.xlsx</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Account Scoring: "Upload a prospect file" = N04_rep_ownership_1_prospects.csv; Score as of 2026-10-20; drop N04_rep_ownership_2_signals.csv. Then send to Micro-segments &amp; NBA and open For Review.</t>
+          <t>Account Scoring: "Upload a prospect file" = N04_rep_ownership.xlsx (reads its "Lead template" sheet); Score as of 2026-10-20; drop the same file on box 2 (reads "Signal template"). Then send to Micro-segments &amp; NBA and open For Review.</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr">

</xml_diff>